<commit_message>
Update EducationCertificationTestCases.xlsx with new test cases
</commit_message>
<xml_diff>
--- a/EducationTestCases.xlsx
+++ b/EducationTestCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muthu\Downloads\qa-dotnet-cucumber-main (2)\qa-dotnet-cucumber-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB7B8B5A-BD78-48C9-9999-B63A1966D84A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A16F35AE-58B7-44FB-8921-CA01A3D1C71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{DED65B8F-8927-44E6-A1B4-A2D58E1FE730}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DED65B8F-8927-44E6-A1B4-A2D58E1FE730}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="421">
   <si>
     <t>TC ID</t>
   </si>
@@ -1292,6 +1292,12 @@
   </si>
   <si>
     <t>Certification</t>
+  </si>
+  <si>
+    <t>"U+0041."</t>
+  </si>
+  <si>
+    <t>"U+0B85"</t>
   </si>
 </sst>
 </file>
@@ -1386,7 +1392,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1401,12 +1407,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1736,7 +1741,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>198</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -1751,7 +1756,7 @@
       <c r="I1" s="4"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>200</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1764,7 +1769,7 @@
       <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>201</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -1777,7 +1782,7 @@
       <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>203</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -1790,7 +1795,7 @@
       <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>204</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -1803,12 +1808,11 @@
       <c r="G5" s="4"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>205</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="4"/>
-      <c r="D6" s="8"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -1816,7 +1820,7 @@
       <c r="I6" s="4"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>206</v>
       </c>
       <c r="B7" s="5"/>
@@ -1829,29 +1833,29 @@
       <c r="I7" s="4"/>
     </row>
     <row r="9" spans="1:9" ht="57.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="10" spans="1:9" s="11" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:9" s="10" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="9" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2867,7 +2871,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>198</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -2882,7 +2886,7 @@
       <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>200</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -2895,7 +2899,7 @@
       <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>201</v>
       </c>
       <c r="B4" s="6" t="s">
@@ -2908,7 +2912,7 @@
       <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>203</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -2921,7 +2925,7 @@
       <c r="G5" s="4"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>204</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -2934,12 +2938,11 @@
       <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>205</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="4"/>
-      <c r="D7" s="8"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -2947,7 +2950,7 @@
       <c r="I7" s="4"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>206</v>
       </c>
       <c r="B8" s="5"/>
@@ -4267,7 +4270,7 @@
         <v>219</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>309</v>
+        <v>419</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>220</v>
@@ -4294,7 +4297,7 @@
         <v>219</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>312</v>
+        <v>420</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>220</v>

</xml_diff>

<commit_message>
Add note/new test case to EducationCertificationTestCases.xlsx
</commit_message>
<xml_diff>
--- a/EducationTestCases.xlsx
+++ b/EducationTestCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muthu\Downloads\qa-dotnet-cucumber-main (2)\qa-dotnet-cucumber-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A16F35AE-58B7-44FB-8921-CA01A3D1C71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5BA21C-BA6E-426E-A57E-6E47ACD02314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DED65B8F-8927-44E6-A1B4-A2D58E1FE730}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{DED65B8F-8927-44E6-A1B4-A2D58E1FE730}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Add CERT-051 edge case: handle 500+ certifications
</commit_message>
<xml_diff>
--- a/EducationTestCases.xlsx
+++ b/EducationTestCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muthu\Downloads\qa-dotnet-cucumber-main (2)\qa-dotnet-cucumber-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5BA21C-BA6E-426E-A57E-6E47ACD02314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565C0747-214A-4999-BA8E-6F5F4D201968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{DED65B8F-8927-44E6-A1B4-A2D58E1FE730}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="425">
   <si>
     <t>TC ID</t>
   </si>
@@ -964,18 +964,12 @@
     <t>Verify system handles Unicode characters in Certification</t>
   </si>
   <si>
-    <t>"高级AI工程师"</t>
-  </si>
-  <si>
     <t>CERT-015</t>
   </si>
   <si>
     <t>Verify system handles Unicode characters in Certified From</t>
   </si>
   <si>
-    <t>"微软"</t>
-  </si>
-  <si>
     <t>CERT-016</t>
   </si>
   <si>
@@ -1298,6 +1292,24 @@
   </si>
   <si>
     <t>"U+0B85"</t>
+  </si>
+  <si>
+    <t>CERT-051</t>
+  </si>
+  <si>
+    <t>Verify system handles extremely large number of certifications</t>
+  </si>
+  <si>
+    <t>1. Add 500+ certifications quickly 2. Save</t>
+  </si>
+  <si>
+    <t>Multiple valid certification data</t>
+  </si>
+  <si>
+    <t>All certifications saved without crash or performance degradation</t>
+  </si>
+  <si>
+    <t>Stress/Destructive</t>
   </si>
 </sst>
 </file>
@@ -2857,7 +2869,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA5B0E3C-39A7-4881-90F7-F42C3FDF53A3}">
-  <dimension ref="A2:I59"/>
+  <dimension ref="A2:I60"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.1796875" customWidth="1"/>
@@ -2890,7 +2902,7 @@
         <v>200</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -3352,7 +3364,7 @@
         <v>170</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>309</v>
+        <v>418</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>220</v>
@@ -3367,10 +3379,10 @@
     </row>
     <row r="24" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>311</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>18</v>
@@ -3379,7 +3391,7 @@
         <v>170</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>312</v>
+        <v>417</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>220</v>
@@ -3394,19 +3406,19 @@
     </row>
     <row r="25" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>82</v>
@@ -3421,22 +3433,22 @@
     </row>
     <row r="26" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>319</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>321</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2" t="s">
@@ -3448,22 +3460,22 @@
     </row>
     <row r="27" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D27" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>324</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>326</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2" t="s">
@@ -3475,7 +3487,7 @@
     </row>
     <row r="28" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>84</v>
@@ -3484,10 +3496,10 @@
         <v>78</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>88</v>
@@ -3502,10 +3514,10 @@
     </row>
     <row r="29" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>212</v>
@@ -3514,10 +3526,10 @@
         <v>222</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2" t="s">
@@ -3529,22 +3541,22 @@
     </row>
     <row r="30" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>336</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>338</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2" t="s">
@@ -3556,22 +3568,22 @@
     </row>
     <row r="31" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2" t="s">
@@ -3583,22 +3595,22 @@
     </row>
     <row r="32" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2" t="s">
@@ -3610,22 +3622,22 @@
     </row>
     <row r="33" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E33" s="2">
         <v>123456</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2" t="s">
@@ -3637,16 +3649,16 @@
     </row>
     <row r="34" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>217</v>
@@ -3664,16 +3676,16 @@
     </row>
     <row r="35" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>242</v>
@@ -3691,16 +3703,16 @@
     </row>
     <row r="36" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>242</v>
@@ -3718,10 +3730,10 @@
     </row>
     <row r="37" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>18</v>
@@ -3745,10 +3757,10 @@
     </row>
     <row r="38" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>18</v>
@@ -3772,10 +3784,10 @@
     </row>
     <row r="39" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>78</v>
@@ -3784,7 +3796,7 @@
         <v>224</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>225</v>
@@ -3799,10 +3811,10 @@
     </row>
     <row r="40" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>99</v>
@@ -3811,7 +3823,7 @@
         <v>227</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>228</v>
@@ -3826,7 +3838,7 @@
     </row>
     <row r="41" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>105</v>
@@ -3838,10 +3850,10 @@
         <v>229</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2" t="s">
@@ -3853,22 +3865,22 @@
     </row>
     <row r="42" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="D42" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="E42" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="F42" s="2" t="s">
         <v>374</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>376</v>
       </c>
       <c r="G42" s="2"/>
       <c r="H42" s="2" t="s">
@@ -3880,7 +3892,7 @@
     </row>
     <row r="43" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>194</v>
@@ -3889,7 +3901,7 @@
         <v>18</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>196</v>
@@ -3907,7 +3919,7 @@
     </row>
     <row r="44" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>231</v>
@@ -3934,22 +3946,22 @@
     </row>
     <row r="45" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>236</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>223</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="G45" s="2"/>
       <c r="H45" s="2" t="s">
@@ -3961,7 +3973,7 @@
     </row>
     <row r="46" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>237</v>
@@ -3988,7 +4000,7 @@
     </row>
     <row r="47" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>255</v>
@@ -4000,7 +4012,7 @@
         <v>256</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>257</v>
@@ -4015,7 +4027,7 @@
     </row>
     <row r="48" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>258</v>
@@ -4027,7 +4039,7 @@
         <v>259</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>257</v>
@@ -4042,16 +4054,16 @@
     </row>
     <row r="49" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E49" s="2">
         <v>2030</v>
@@ -4069,22 +4081,22 @@
     </row>
     <row r="50" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="G50" s="2"/>
       <c r="H50" s="2" t="s">
@@ -4096,22 +4108,22 @@
     </row>
     <row r="51" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2" t="s">
@@ -4123,22 +4135,22 @@
     </row>
     <row r="52" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G52" s="2"/>
       <c r="H52" s="2" t="s">
@@ -4150,22 +4162,22 @@
     </row>
     <row r="53" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>212</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>223</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="G53" s="2"/>
       <c r="H53" s="2" t="s">
@@ -4177,7 +4189,7 @@
     </row>
     <row r="54" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>84</v>
@@ -4186,10 +4198,10 @@
         <v>78</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>88</v>
@@ -4204,16 +4216,16 @@
     </row>
     <row r="55" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>250</v>
@@ -4231,19 +4243,19 @@
     </row>
     <row r="56" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>249</v>
@@ -4258,10 +4270,10 @@
     </row>
     <row r="57" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>18</v>
@@ -4270,7 +4282,7 @@
         <v>219</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>220</v>
@@ -4285,10 +4297,10 @@
     </row>
     <row r="58" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>18</v>
@@ -4297,7 +4309,7 @@
         <v>219</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>220</v>
@@ -4312,22 +4324,22 @@
     </row>
     <row r="59" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>238</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="G59" s="2"/>
       <c r="H59" s="2" t="s">
@@ -4335,6 +4347,33 @@
       </c>
       <c r="I59" s="2" t="s">
         <v>230</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>